<commit_message>
Added acknowledgements change and changed video
</commit_message>
<xml_diff>
--- a/Questionnaire_data/TS_advanced_mapping_v2 (1).xlsx
+++ b/Questionnaire_data/TS_advanced_mapping_v2 (1).xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sadiqkhawaja/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sadiqkhawaja/Desktop/PhD/CVD_RiskStrat_WebApp-merge-interface2/Questionnaire_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{441D5E66-E496-354B-89FA-311FAA7DD379}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C508873D-7148-9B47-88B1-8AD07DC0A77A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17380" xr2:uid="{5A91DBF8-AF45-5544-993E-463958C0A548}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" xr2:uid="{5A91DBF8-AF45-5544-993E-463958C0A548}"/>
   </bookViews>
   <sheets>
     <sheet name="TS_advanced_mapping_v2" sheetId="1" r:id="rId1"/>

</xml_diff>